<commit_message>
feat: đồng bộ web với tài liệu nhóm — 5 đèn thật, QR chỉ ở thiệp cảm ơn, nội dung trang chủ (D-104)
</commit_message>
<xml_diff>
--- a/docs/client-checklist/LAMVI-task-tracker-client.xlsx
+++ b/docs/client-checklist/LAMVI-task-tracker-client.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task tracker" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Task tracker'!$A$1:$L$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Task tracker'!$A$1:$L$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Task tracker'!A2:A93)</f>
+        <f>COUNTA('Task tracker'!A2:A98)</f>
         <v/>
       </c>
     </row>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIF('Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIFS('Task tracker'!E2:E93,"🔴 Chặn go-live",'Task tracker'!G2:G93,"&lt;&gt;Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E98,"🔴 Chặn go-live",'Task tracker'!G2:G98,"&lt;&gt;Xong")</f>
         <v/>
       </c>
     </row>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>SUMPRODUCT(('Task tracker'!I2:I93&lt;&gt;"")*('Task tracker'!I2:I93&lt;TODAY())*('Task tracker'!G2:G93&lt;&gt;"Xong"))</f>
+        <f>SUMPRODUCT(('Task tracker'!I2:I98&lt;&gt;"")*('Task tracker'!I2:I98&lt;TODAY())*('Task tracker'!G2:G98&lt;&gt;"Xong"))</f>
         <v/>
       </c>
     </row>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF('Task tracker'!G2:G93,A11)</f>
+        <f>COUNTIF('Task tracker'!G2:G98,A11)</f>
         <v/>
       </c>
     </row>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF('Task tracker'!G2:G93,A12)</f>
+        <f>COUNTIF('Task tracker'!G2:G98,A12)</f>
         <v/>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF('Task tracker'!G2:G93,A13)</f>
+        <f>COUNTIF('Task tracker'!G2:G98,A13)</f>
         <v/>
       </c>
     </row>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIF('Task tracker'!G2:G93,A14)</f>
+        <f>COUNTIF('Task tracker'!G2:G98,A14)</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIF('Task tracker'!G2:G93,A15)</f>
+        <f>COUNTIF('Task tracker'!G2:G98,A15)</f>
         <v/>
       </c>
     </row>
@@ -690,11 +690,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF('Task tracker'!E2:E93,A18)</f>
+        <f>COUNTIF('Task tracker'!E2:E98,A18)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS('Task tracker'!E2:E93,A18,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E98,A18,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -705,11 +705,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF('Task tracker'!E2:E93,A19)</f>
+        <f>COUNTIF('Task tracker'!E2:E98,A19)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS('Task tracker'!E2:E93,A19,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E98,A19,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -720,11 +720,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIF('Task tracker'!E2:E93,A20)</f>
+        <f>COUNTIF('Task tracker'!E2:E98,A20)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS('Task tracker'!E2:E93,A20,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E98,A20,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -757,11 +757,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Task tracker'!B2:B93,A24)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A24)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS('Task tracker'!B2:B93,A24,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A24,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D24">
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIF('Task tracker'!B2:B93,A25)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A25)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS('Task tracker'!B2:B93,A25,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A25,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D25">
@@ -795,11 +795,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIF('Task tracker'!B2:B93,A26)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A26)</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS('Task tracker'!B2:B93,A26,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A26,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D26">
@@ -814,11 +814,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIF('Task tracker'!B2:B93,A27)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A27)</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS('Task tracker'!B2:B93,A27,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A27,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D27">
@@ -833,11 +833,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIF('Task tracker'!B2:B93,A28)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A28)</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS('Task tracker'!B2:B93,A28,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A28,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D28">
@@ -852,11 +852,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIF('Task tracker'!B2:B93,A29)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A29)</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS('Task tracker'!B2:B93,A29,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A29,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D29">
@@ -871,11 +871,11 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIF('Task tracker'!B2:B93,A30)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A30)</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS('Task tracker'!B2:B93,A30,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A30,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D30">
@@ -890,11 +890,11 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIF('Task tracker'!B2:B93,A31)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A31)</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS('Task tracker'!B2:B93,A31,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A31,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D31">
@@ -909,11 +909,11 @@
         </is>
       </c>
       <c r="B32">
-        <f>COUNTIF('Task tracker'!B2:B93,A32)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A32)</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS('Task tracker'!B2:B93,A32,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A32,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D32">
@@ -928,11 +928,11 @@
         </is>
       </c>
       <c r="B33">
-        <f>COUNTIF('Task tracker'!B2:B93,A33)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A33)</f>
         <v/>
       </c>
       <c r="C33">
-        <f>COUNTIFS('Task tracker'!B2:B93,A33,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A33,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D33">
@@ -947,11 +947,11 @@
         </is>
       </c>
       <c r="B34">
-        <f>COUNTIF('Task tracker'!B2:B93,A34)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A34)</f>
         <v/>
       </c>
       <c r="C34">
-        <f>COUNTIFS('Task tracker'!B2:B93,A34,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A34,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D34">
@@ -966,11 +966,11 @@
         </is>
       </c>
       <c r="B35">
-        <f>COUNTIF('Task tracker'!B2:B93,A35)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A35)</f>
         <v/>
       </c>
       <c r="C35">
-        <f>COUNTIFS('Task tracker'!B2:B93,A35,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A35,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D35">
@@ -985,11 +985,11 @@
         </is>
       </c>
       <c r="B36">
-        <f>COUNTIF('Task tracker'!B2:B93,A36)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A36)</f>
         <v/>
       </c>
       <c r="C36">
-        <f>COUNTIFS('Task tracker'!B2:B93,A36,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A36,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D36">
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="B37">
-        <f>COUNTIF('Task tracker'!B2:B93,A37)</f>
+        <f>COUNTIF('Task tracker'!B2:B98,A37)</f>
         <v/>
       </c>
       <c r="C37">
-        <f>COUNTIFS('Task tracker'!B2:B93,A37,'Task tracker'!G2:G93,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B98,A37,'Task tracker'!G2:G98,"Xong")</f>
         <v/>
       </c>
       <c r="D37">
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1543,14 +1543,18 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
       <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>13/10: 5 đèn thật đã lên web (tên, mô tả, thông số, giá tạm). Duyệt tab "Sản phẩm" trong file nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1585,14 +1589,18 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="10" t="n"/>
       <c r="J13" s="10" t="n"/>
       <c r="K13" s="9" t="n"/>
-      <c r="L13" s="9" t="n"/>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã điền 4/6 thông số (kích thước, chất liệu, nguồn sáng, thời gian làm). Thiếu cân nặng, bảo quản → xem 2.7</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1665,14 +1673,18 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="10" t="n"/>
       <c r="J15" s="10" t="n"/>
       <c r="K15" s="9" t="n"/>
-      <c r="L15" s="9" t="n"/>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Không còn áp dụng: không có bộ Sum Vầy (D-104)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1715,22 +1727,22 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Bộ sưu tập</t>
+          <t>Sản phẩm</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Điền nội dung mỗi bộ sưu tập</t>
+          <t>Chốt giá thật từng mẫu trong 5 đèn</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Tab "Bộ sưu tập": tên, mô tả, câu chuyện; ảnh bìa ngang ≥1600px</t>
+          <t>Hiện đang là giá tạm 1.400.000đ cho cả 5 (trung điểm 1,3–1,5 triệu của báo cáo, chưa kiểm chứng)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1740,7 +1752,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>§3</t>
+          <t>§2</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
@@ -1757,32 +1769,32 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Bộ sưu tập</t>
+          <t>Sản phẩm</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Chốt có thêm category/bộ lọc khác không</t>
+          <t>Gửi cân nặng và cách bảo quản của đèn</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Theo dịp (Tết, Trung thu, tân gia…), theo không gian (bàn trà, phòng ngủ…), theo giá</t>
+          <t>Hai trong 6 thông số còn trống; xác nhận kích thước chốt (báo cáo ghi 12×12×20 cm là prototype)</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>§3</t>
+          <t>§2</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -1799,22 +1811,22 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Bộ sưu tập</t>
+          <t>Sản phẩm</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Viết nội dung phần thưởng cốt truyện cho Gallery / chăn Đông Hồ</t>
+          <t>Viết mô tả dài / câu chuyện cho từng đèn</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Và xác nhận còn muốn giữ tính năng này</t>
+          <t>Content Plan đã có bài dài cho 5 đèn; web hiện chỉ có mô tả 1 câu — cho biết dùng nguyên bài hay rút gọn</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1824,7 +1836,7 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>§3</t>
+          <t>§2</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -1841,22 +1853,22 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Trang chủ</t>
+          <t>Bộ sưu tập</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Duyệt/sửa Hero (HOME-02) + gửi ảnh hoặc video hero thật</t>
+          <t>Điền nội dung mỗi bộ sưu tập</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận "làng nghề trăm năm" đúng sự thật</t>
+          <t>Tab "Bộ sưu tập": tên, mô tả, câu chuyện; ảnh bìa ngang ≥1600px</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1866,45 +1878,53 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>§4</t>
+          <t>§3</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="10" t="n"/>
       <c r="J20" s="10" t="n"/>
       <c r="K20" s="9" t="n"/>
-      <c r="L20" s="9" t="n"/>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>13/10: 1 bộ "Bộ sưu tập đầu tiên" + câu chuyện bộ do dev soạn từ Content Plan</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Trang chủ</t>
+          <t>Bộ sưu tập</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Duyệt dải chữ chạy (HOME-03)</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr"/>
+          <t>Chốt có thêm category/bộ lọc khác không</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Theo dịp (Tết, Trung thu, tân gia…), theo không gian (bàn trà, phòng ngủ…), theo giá</t>
+        </is>
+      </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>§4</t>
+          <t>§3</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -1921,32 +1941,32 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Trang chủ</t>
+          <t>Bộ sưu tập</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Gửi số liệu thật + câu chuyện làng nghề (HOME-04)</t>
+          <t>Viết nội dung phần thưởng cốt truyện cho Gallery / chăn Đông Hồ</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>79+ năm, 10 nghệ nhân hiện là số MẪU</t>
+          <t>Và xác nhận còn muốn giữ tính năng này</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>§4</t>
+          <t>§3</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -1963,7 +1983,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -1973,12 +1993,12 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Khối Nghệ nhân (HOME-05): gửi nhân vật thật hoặc bỏ khối</t>
+          <t>Duyệt/sửa Hero (HOME-02) + gửi ảnh hoặc video hero thật</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Tên, ảnh chân dung, câu nói, 32 năm / 4.000+ đèn là mẫu; cần văn bản đồng ý của nghệ nhân</t>
+          <t>Xác nhận "làng nghề trăm năm" đúng sự thật</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -2005,7 +2025,7 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -2015,13 +2035,13 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Duyệt câu giới thiệu bộ sưu tập (HOME-06)</t>
+          <t>Duyệt dải chữ chạy (HOME-03)</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -2043,7 +2063,7 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -2053,13 +2073,17 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Lookbook (HOME-07): gửi ảnh thật + chốt 5 tên màu</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr"/>
+          <t>Gửi số liệu thật + câu chuyện làng nghề (HOME-04)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>79+ năm, 10 nghệ nhân hiện là số MẪU</t>
+        </is>
+      </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -2069,19 +2093,23 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="10" t="n"/>
       <c r="J25" s="10" t="n"/>
       <c r="K25" s="9" t="n"/>
-      <c r="L25" s="9" t="n"/>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã thay số mẫu bằng 5 đèn / 3 chặng / 1 lời chúc. Cần câu chuyện làng nghề thật</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
@@ -2091,13 +2119,17 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Hành trình thủ công (HOME-08): xác nhận 4 bước + ảnh/video từng bước</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr"/>
+          <t>Khối Nghệ nhân (HOME-05): gửi nhân vật thật hoặc bỏ khối</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Tên, ảnh chân dung, câu nói, 32 năm / 4.000+ đèn là mẫu; cần văn bản đồng ý của nghệ nhân</t>
+        </is>
+      </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -2107,19 +2139,23 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="10" t="n"/>
       <c r="J26" s="10" t="n"/>
       <c r="K26" s="9" t="n"/>
-      <c r="L26" s="9" t="n"/>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã dùng tên Nghệ nhân Ưu tú Nguyễn Hữu Quả, bỏ câu trích + số liệu mẫu. Cần ảnh + đồng ý → xem 8.11</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -2129,14 +2165,10 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Duyệt khối Trải nghiệm QR (HOME-09)</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Nhất là câu thời hạn lưu 30 ngày</t>
-        </is>
-      </c>
+          <t>Duyệt câu giới thiệu bộ sưu tập (HOME-06)</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr"/>
       <c r="E27" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2161,7 +2193,7 @@
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
@@ -2171,17 +2203,13 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Testimonials (HOME-10): gửi đánh giá thật + đồng ý của người viết, hoặc bỏ</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Hiện đang ẩn</t>
-        </is>
-      </c>
+          <t>Lookbook (HOME-07): gửi ảnh thật + chốt 5 tên màu</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr"/>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -2191,19 +2219,23 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="10" t="n"/>
       <c r="J28" s="10" t="n"/>
       <c r="K28" s="9" t="n"/>
-      <c r="L28" s="9" t="n"/>
+      <c r="L28" s="9" t="inlineStr">
+        <is>
+          <t>13/10: lookbook = 5 tên đèn. Cần ảnh thật</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -2213,17 +2245,13 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Duyệt 5 FAQ + thêm câu hỏi thực tế khách hay hỏi (HOME-11)</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Tab "FAQ"</t>
-        </is>
-      </c>
+          <t>Hành trình thủ công (HOME-08): xác nhận 4 bước + ảnh/video từng bước</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr"/>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -2233,19 +2261,23 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="10" t="n"/>
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="9" t="n"/>
-      <c r="L29" s="9" t="n"/>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t>13/10: 4 bước đã đổi theo Content Plan. Cần xác nhận + ảnh/video</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>4.11</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
@@ -2255,10 +2287,14 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Duyệt tiêu đề/mô tả SEO hiện trên Google</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr"/>
+          <t>Duyệt khối Trải nghiệm QR (HOME-09)</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Nhất là câu thời hạn lưu 30 ngày</t>
+        </is>
+      </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2271,19 +2307,23 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="10" t="n"/>
       <c r="J30" s="10" t="n"/>
       <c r="K30" s="9" t="n"/>
-      <c r="L30" s="9" t="n"/>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã sửa QR chỉ ở thiệp cảm ơn (D-104)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -2293,10 +2333,14 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Chốt giữ hay bỏ form newsletter (G-11)</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr"/>
+          <t>Testimonials (HOME-10): gửi đánh giá thật + đồng ý của người viết, hoặc bỏ</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Hiện đang ẩn</t>
+        </is>
+      </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
           <t>🟡 Làm sau được</t>
@@ -2321,59 +2365,63 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Các trang khác</t>
+          <t>Trang chủ</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Cửa hàng / Chi tiết sản phẩm / Bộ sưu tập</t>
+          <t>Duyệt 5 FAQ + thêm câu hỏi thực tế khách hay hỏi (HOME-11)</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Tab "Nội dung web"</t>
+          <t>Tab "FAQ"</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>§5</t>
+          <t>§4</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="10" t="n"/>
       <c r="J32" s="10" t="n"/>
       <c r="K32" s="9" t="n"/>
-      <c r="L32" s="9" t="n"/>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>13/10: FAQ 9 câu (thêm 4 câu). Cần thêm câu hỏi thực tế</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>4.11</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Các trang khác</t>
+          <t>Trang chủ</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Giỏ hàng / Thanh toán / Đơn hàng</t>
+          <t>Duyệt tiêu đề/mô tả SEO hiện trên Google</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr"/>
@@ -2384,7 +2432,7 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>§5</t>
+          <t>§4</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
@@ -2401,28 +2449,28 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Các trang khác</t>
+          <t>Trang chủ</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Đăng nhập / Đăng ký / Quên mật khẩu + gửi ảnh nền thương hiệu</t>
+          <t>Chốt giữ hay bỏ form newsletter (G-11)</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr"/>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>§5</t>
+          <t>§4</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -2439,7 +2487,7 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -2449,12 +2497,12 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ trang người nhận mở lời chúc (QR-GIFT)</t>
+          <t>Duyệt chữ Cửa hàng / Chi tiết sản phẩm / Bộ sưu tập</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Điểm chạm cảm xúc nhất — nên do copywriter viết</t>
+          <t>Tab "Nội dung web"</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -2481,7 +2529,7 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -2491,7 +2539,7 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Liên hệ, 404, bảo trì</t>
+          <t>Duyệt chữ Giỏ hàng / Thanh toán / Đơn hàng</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr"/>
@@ -2519,7 +2567,7 @@
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -2529,14 +2577,10 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Duyệt tên các trạng thái đơn hàng</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Chờ thanh toán, Đang làm, Đã đóng gói, Đã gửi, Đã giao, Đã huỷ, Hoàn tiền</t>
-        </is>
-      </c>
+          <t>Duyệt chữ Đăng nhập / Đăng ký / Quên mật khẩu + gửi ảnh nền thương hiệu</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr"/>
       <c r="E37" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2561,22 +2605,22 @@
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Mây (AI)</t>
+          <t>Các trang khác</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Chốt tính cách &amp; giọng nói của Mây</t>
+          <t>Duyệt chữ trang người nhận mở lời chúc (QR-GIFT)</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Xưng hô, từ nên/cấm dùng, độ dài câu trả lời</t>
+          <t>Điểm chạm cảm xúc nhất — nên do copywriter viết</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2586,7 +2630,7 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>§6</t>
+          <t>§5</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -2603,32 +2647,28 @@
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Mây (AI)</t>
+          <t>Các trang khác</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Viết kho kiến thức cho Mây (≥30 câu FAQ)</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Chất liệu, quy trình, bảo quản, an toàn, quà doanh nghiệp, in logo…</t>
-        </is>
-      </c>
+          <t>Duyệt chữ Liên hệ, 404, bảo trì</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr"/>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>§6</t>
+          <t>§5</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -2645,20 +2685,24 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Mây (AI)</t>
+          <t>Các trang khác</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Danh sách chủ đề Mây không được trả lời / phải chuyển nhân viên</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr"/>
+          <t>Duyệt tên các trạng thái đơn hàng</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Chờ thanh toán, Đang làm, Đã đóng gói, Đã gửi, Đã giao, Đã huỷ, Hoàn tiền</t>
+        </is>
+      </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2666,7 +2710,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>§6</t>
+          <t>§5</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
@@ -2683,7 +2727,7 @@
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -2693,17 +2737,17 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Cung cấp kênh chuyển nhân viên + giờ trực</t>
+          <t>Chốt tính cách &amp; giọng nói của Mây</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Zalo / hotline / email</t>
+          <t>Xưng hô, từ nên/cấm dùng, độ dài câu trả lời</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -2725,7 +2769,7 @@
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
@@ -2735,17 +2779,17 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Duyệt câu báo lỗi, câu gợi ý, câu chào, tour 5 bước</t>
+          <t>Viết kho kiến thức cho Mây (≥30 câu FAQ)</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Tab "Mây" và "Nội dung web"</t>
+          <t>Chất liệu, quy trình, bảo quản, an toàn, quà doanh nghiệp, in logo…</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -2755,19 +2799,23 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="10" t="n"/>
       <c r="J42" s="10" t="n"/>
       <c r="K42" s="9" t="n"/>
-      <c r="L42" s="9" t="n"/>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>13/10: FAQ mới 9 câu — Mây dùng FAQ làm kiến thức</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -2777,17 +2825,13 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Chốt hạn mức &amp; ngân sách OpenAI</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>Hiện 20 USD/tháng; 20/50/100 tin nhắn</t>
-        </is>
-      </c>
+          <t>Danh sách chủ đề Mây không được trả lời / phải chuyển nhân viên</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr"/>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -2809,7 +2853,7 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
@@ -2819,10 +2863,14 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Pháp chế duyệt thông báo xử lý dữ liệu ở nước ngoài + quyền xoá lịch sử chat (I-15)</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr"/>
+          <t>Cung cấp kênh chuyển nhân viên + giờ trực</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Zalo / hotline / email</t>
+        </is>
+      </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -2847,70 +2895,78 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Lô đèn &amp; QR</t>
+          <t>Mây (AI)</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Quay &amp; gửi video quy trình cho lô đầu tiên</t>
+          <t>Duyệt câu báo lỗi, câu gợi ý, câu chào, tour 5 bước</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Mã lô, ngày làm, tiêu đề VI/EN/ZH, câu chuyện, file MP4/WebM/MOV ≤500 MB</t>
+          <t>Tab "Mây" và "Nội dung web"</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>§7</t>
+          <t>§6</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="10" t="n"/>
       <c r="J45" s="10" t="n"/>
       <c r="K45" s="9" t="n"/>
-      <c r="L45" s="9" t="n"/>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>13/10: câu tour về QR đã sửa theo D-104</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Lô đèn &amp; QR</t>
+          <t>Mây (AI)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Chốt quy tắc đặt mã lô + quy trình khắc/in QR lên đèn</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr"/>
+          <t>Chốt hạn mức &amp; ngân sách OpenAI</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Hiện 20 USD/tháng; 20/50/100 tin nhắn</t>
+        </is>
+      </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>§7</t>
+          <t>§6</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
@@ -2927,32 +2983,28 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Lô đèn &amp; QR</t>
+          <t>Mây (AI)</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Thiết kế thiệp cảm ơn có mã QR</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Kích thước, mặt trước/sau, mẫu viết tay hay in</t>
-        </is>
-      </c>
+          <t>Pháp chế duyệt thông báo xử lý dữ liệu ở nước ngoài + quyền xoá lịch sử chat (I-15)</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr"/>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>§7</t>
+          <t>§6</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
@@ -2969,7 +3021,7 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
@@ -2979,13 +3031,17 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận chính sách lưu trữ lời chúc (30 ngày giọng nói/video)</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr"/>
+          <t>Quay &amp; gửi video quy trình cho lô đầu tiên</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Mã lô, ngày làm, tiêu đề VI/EN/ZH, câu chuyện, file MP4/WebM/MOV ≤500 MB</t>
+        </is>
+      </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -3007,7 +3063,7 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -3017,14 +3073,10 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Trả lời Q-12, Q-14, Q-25, Q-27, Q-29, Q-33</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Phí thiệp; admin xem lời chúc; QR đơn tự mua; xem trước; lời chúc không phải tiếng Việt; PIN</t>
-        </is>
-      </c>
+          <t>Chốt quy tắc đặt mã lô + quy trình in thiệp có QR (không khắc lên đèn)</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr"/>
       <c r="E49" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -3032,7 +3084,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>§7/§13</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
@@ -3049,28 +3101,32 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Gửi tên pháp nhân + tên thương mại</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr"/>
+          <t>Thiết kế thiệp cảm ơn có mã QR</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Kích thước, mặt trước/sau, mẫu viết tay hay in</t>
+        </is>
+      </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
@@ -3087,28 +3143,28 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Gửi MST / số ĐKKD, ngày cấp, nơi cấp</t>
+          <t>Xác nhận chính sách lưu trữ lời chúc (30 ngày giọng nói/video)</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr"/>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
@@ -3125,28 +3181,32 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Gửi địa chỉ trụ sở + địa chỉ xưởng</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr"/>
+          <t>Trả lời Q-12, Q-14, Q-25, Q-27, Q-29, Q-33</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Phí thiệp; admin xem lời chúc; QR đơn tự mua; xem trước; lời chúc không phải tiếng Việt; PIN</t>
+        </is>
+      </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7/§13</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -3163,28 +3223,32 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Gửi hotline, Zalo, email hỗ trợ, giờ làm việc</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr"/>
+          <t>Quyết định trang kể chuyện theo từng mẫu đèn (QR trên thiệp)</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Content Plan 30/10: QR mở nội dung riêng của mẫu (artwork, chi tiết) rồi mới tới lời chúc. Web chưa có (G-108) — chốt phạm vi + nội dung</t>
+        </is>
+      </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
@@ -3201,7 +3265,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
@@ -3211,17 +3275,13 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Gửi link mạng xã hội</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>Facebook, Instagram, TikTok, Zalo OA, YouTube (https)</t>
-        </is>
-      </c>
+          <t>Gửi tên pháp nhân + tên thương mại</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr"/>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -3243,7 +3303,7 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>8.6</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -3253,14 +3313,10 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Thông báo website TMĐT với Bộ Công Thương + gửi link xác nhận</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>online.gov.vn (Q-42)</t>
-        </is>
-      </c>
+          <t>Gửi MST / số ĐKKD, ngày cấp, nơi cấp</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr"/>
       <c r="E55" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3285,7 +3341,7 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
@@ -3295,14 +3351,10 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Chỉ định người đại diện / bên kiểm soát dữ liệu + email nhận yêu cầu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>Q-40</t>
-        </is>
-      </c>
+          <t>Gửi địa chỉ trụ sở + địa chỉ xưởng</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr"/>
       <c r="E56" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3327,7 +3379,7 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -3337,7 +3389,7 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Chốt tên miền chính thức + cấp quyền DNS</t>
+          <t>Gửi hotline, Zalo, email hỗ trợ, giờ làm việc</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr"/>
@@ -3365,7 +3417,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
@@ -3375,17 +3427,17 @@
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Pháp chế duyệt 5 trang chính sách + banner cookie/GA</t>
+          <t>Gửi link mạng xã hội</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Q-40, Q-42, Q-43</t>
+          <t>Facebook, Instagram, TikTok, Zalo OA, YouTube (https)</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -3407,7 +3459,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>8.10</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -3417,10 +3469,14 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Giấy phép ảnh: tư liệu Đông Hồ (Q-36), ảnh nghệ nhân, ảnh sản phẩm</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr"/>
+          <t>Thông báo website TMĐT với Bộ Công Thương + gửi link xác nhận</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>online.gov.vn (Q-42)</t>
+        </is>
+      </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3445,22 +3501,22 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Chốt phí ship + ngưỡng freeship</t>
+          <t>Chỉ định người đại diện / bên kiểm soát dữ liệu + email nhận yêu cầu dữ liệu</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>Hiện 30.000đ, miễn phí từ 1.000.000đ (giả định)</t>
+          <t>Q-40</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -3470,7 +3526,7 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -3487,17 +3543,17 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Chốt đơn vị vận chuyển, thời gian giao theo vùng, vùng không giao</t>
+          <t>Chốt tên miền chính thức + cấp quyền DNS</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr"/>
@@ -3508,7 +3564,7 @@
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
@@ -3525,20 +3581,24 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận thời gian làm đèn (5–7 ngày làm việc?)</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr"/>
+          <t>Pháp chế duyệt 5 trang chính sách + banner cookie/GA</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Q-40, Q-42, Q-43</t>
+        </is>
+      </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3546,7 +3606,7 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
@@ -3563,24 +3623,20 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>8.10</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận VAT 10% + cách xuất hoá đơn điện tử</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>Hệ thống chưa có xuất hoá đơn</t>
-        </is>
-      </c>
+          <t>Giấy phép ảnh: tư liệu Đông Hồ (Q-36), ảnh nghệ nhân, ảnh sản phẩm</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr"/>
       <c r="E63" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3588,7 +3644,7 @@
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
@@ -3605,20 +3661,24 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Mở tài khoản payOS + quyết định COD (giới hạn giá trị? Q-37)</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr"/>
+          <t>Gửi ảnh chân dung + văn bản đồng ý của Nghệ nhân Ưu tú Nguyễn Hữu Quả</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Web đã dùng tên thật theo Content Plan; ảnh vẫn là hình minh hoạ. Không đưa phần "Tài liệu tham khảo" trích nguồn ngoài lên web khi chưa xin phép</t>
+        </is>
+      </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3626,7 +3686,7 @@
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§4/§8</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
@@ -3643,7 +3703,7 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
@@ -3653,17 +3713,17 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Chốt chính sách đổi trả còn mở</t>
+          <t>Chốt phí ship + ngưỡng freeship</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>Q-06 trả 1 đèn trong bộ; Q-20 mức hoàn khi huỷ đơn đã thanh toán; thời gian hoàn tiền; ai chịu phí ship đổi trả</t>
+          <t>Hiện 30.000đ, miễn phí từ 1.000.000đ (giả định)</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -3685,7 +3745,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
@@ -3695,13 +3755,13 @@
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Lên danh sách coupon ra mắt</t>
+          <t>Chốt đơn vị vận chuyển, thời gian giao theo vùng, vùng không giao</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr"/>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -3723,7 +3783,7 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
@@ -3733,13 +3793,13 @@
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Chốt có bán quà doanh nghiệp / in logo không</t>
+          <t>Xác nhận thời gian làm đèn (5–7 ngày làm việc?)</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr"/>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -3761,7 +3821,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
@@ -3771,13 +3831,17 @@
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Mô tả quy trình xử lý đơn nội bộ (ai làm gì, khi nào đổi trạng thái)</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr"/>
+          <t>Xác nhận VAT 10% + cách xuất hoá đơn điện tử</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Hệ thống chưa có xuất hoá đơn</t>
+        </is>
+      </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -3799,7 +3863,7 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>9.10</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
@@ -3809,13 +3873,13 @@
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Chốt chính sách bảo hành (nếu có)</t>
+          <t>Mở tài khoản payOS + quyết định COD (giới hạn giá trị? Q-37)</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr"/>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -3837,22 +3901,22 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Duyệt nội dung email giao dịch</t>
+          <t>Chốt chính sách đổi trả còn mở</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Tab "Email"</t>
+          <t>Q-06 trả 1 đèn trong bộ; Q-20 mức hoàn khi huỷ đơn đã thanh toán; thời gian hoàn tiền; ai chịu phí ship đổi trả</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -3862,7 +3926,7 @@
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>§10</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
@@ -3879,32 +3943,28 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Chọn địa chỉ gửi + xác minh tên miền gửi (SPF/DKIM)</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>Cần quyền DNS</t>
-        </is>
-      </c>
+          <t>Lên danh sách coupon ra mắt</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr"/>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>§10</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
@@ -3921,17 +3981,17 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Chốt có SMS/Zalo thông báo đơn không (Q-24)</t>
+          <t>Chốt có bán quà doanh nghiệp / in logo không</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr"/>
@@ -3942,7 +4002,7 @@
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>§10</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G72" s="9" t="inlineStr">
@@ -3959,28 +4019,28 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Tên miền + DNS</t>
+          <t>Mô tả quy trình xử lý đơn nội bộ (ai làm gì, khi nào đổi trạng thái)</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr"/>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
@@ -3997,28 +4057,28 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>9.10</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Tạo / cấp quyền Vercel</t>
+          <t>Chốt chính sách bảo hành (nếu có)</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr"/>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G74" s="9" t="inlineStr">
@@ -4035,28 +4095,32 @@
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Tạo project Supabase production (gói phù hợp, có sao lưu)</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr"/>
+          <t>Duyệt nội dung email giao dịch</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Tab "Email"</t>
+        </is>
+      </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§10</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
@@ -4073,22 +4137,22 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Đăng ký payOS, lấy Client ID / API Key / Checksum Key</t>
+          <t>Chọn địa chỉ gửi + xác minh tên miền gửi (SPF/DKIM)</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>Chia sẻ khoá qua kênh an toàn</t>
+          <t>Cần quyền DNS</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -4098,7 +4162,7 @@
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§10</t>
         </is>
       </c>
       <c r="G76" s="9" t="inlineStr">
@@ -4115,28 +4179,28 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Resend hoặc Brevo</t>
+          <t>Chốt có SMS/Zalo thông báo đơn không (Q-24)</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr"/>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§10</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
@@ -4153,7 +4217,7 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
@@ -4163,13 +4227,13 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Google Analytics 4: Measurement ID + quyền Viewer</t>
+          <t>Tên miền + DNS</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr"/>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
@@ -4191,7 +4255,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
@@ -4201,17 +4265,13 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Google Cloud OAuth (đăng nhập bằng Google)</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>Cần logo + chính sách riêng tư + miền thật</t>
-        </is>
-      </c>
+          <t>Tạo / cấp quyền Vercel</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr"/>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -4233,7 +4293,7 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
@@ -4243,13 +4303,13 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>OpenAI API key + hạn mức chi tiêu</t>
+          <t>Tạo project Supabase production (gói phù hợp, có sao lưu)</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr"/>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -4271,7 +4331,7 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>11.9</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
@@ -4281,13 +4341,17 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Google Search Console (xác minh tên miền)</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr"/>
+          <t>Đăng ký payOS, lấy Client ID / API Key / Checksum Key</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Chia sẻ khoá qua kênh an toàn</t>
+        </is>
+      </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
@@ -4309,7 +4373,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>11.10</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
@@ -4319,17 +4383,13 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Quyết định gắn pixel quảng cáo (Facebook/TikTok)</t>
-        </is>
-      </c>
-      <c r="D82" s="8" t="inlineStr">
-        <is>
-          <t>Cần cập nhật banner cookie</t>
-        </is>
-      </c>
+          <t>Tài khoản Resend hoặc Brevo</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr"/>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
@@ -4351,24 +4411,20 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Dịch thuật</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Chốt có bán cho khách EN / ZH không</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="inlineStr">
-        <is>
-          <t>Nếu không thì có thể ẩn để giảm công duy trì</t>
-        </is>
-      </c>
+          <t>Google Analytics 4: Measurement ID + quyền Viewer</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr"/>
       <c r="E83" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -4376,7 +4432,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G83" s="9" t="inlineStr">
@@ -4393,32 +4449,32 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Dịch thuật</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Thuê người bản ngữ duyệt bản EN / ZH</t>
+          <t>Google Cloud OAuth (đăng nhập bằng Google)</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>Tên sản phẩm, câu chuyện, chính sách, email</t>
+          <t>Cần logo + chính sách riêng tư + miền thật</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G84" s="9" t="inlineStr">
@@ -4435,28 +4491,28 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>11.8</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Dịch thuật</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Chốt quy ước tên riêng khi dịch (giấy dó, Đông Hồ, Mây)</t>
+          <t>OpenAI API key + hạn mức chi tiêu</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr"/>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G85" s="9" t="inlineStr">
@@ -4473,32 +4529,28 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>11.9</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Quyết định nghiệp vụ</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Q-41: cho phép mua không cần tài khoản (guest checkout)?</t>
-        </is>
-      </c>
-      <c r="D86" s="8" t="inlineStr">
-        <is>
-          <t>Thay đổi lớn — cần quyết rõ</t>
-        </is>
-      </c>
+          <t>Google Search Console (xác minh tên miền)</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr"/>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>§13</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G86" s="9" t="inlineStr">
@@ -4515,28 +4567,32 @@
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>11.10</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>Quyết định nghiệp vụ</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Q-35: đăng ký email đã tồn tại báo "đã đăng ký" hay "kiểm tra email"?</t>
-        </is>
-      </c>
-      <c r="D87" s="8" t="inlineStr"/>
+          <t>Quyết định gắn pixel quảng cáo (Facebook/TikTok)</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Cần cập nhật banner cookie</t>
+        </is>
+      </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>§13</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G87" s="9" t="inlineStr">
@@ -4553,32 +4609,32 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>Quyết định nghiệp vụ</t>
+          <t>Dịch thuật</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Q-21, Q-23, Q-38 và KPI mong muốn</t>
+          <t>Chốt có bán cho khách EN / ZH không</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>Phiếu giao không in giá; testimonial; ngưỡng chống spam; KPI</t>
+          <t>Nếu không thì có thể ẩn để giảm công duy trì</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>§13</t>
+          <t>§12</t>
         </is>
       </c>
       <c r="G88" s="9" t="inlineStr">
@@ -4595,28 +4651,32 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Dịch thuật</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Gửi danh sách người dùng admin (email, vai trò admin/IT)</t>
-        </is>
-      </c>
-      <c r="D89" s="8" t="inlineStr"/>
+          <t>Thuê người bản ngữ duyệt bản EN / ZH</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Tên sản phẩm, câu chuyện, chính sách, email</t>
+        </is>
+      </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§12</t>
         </is>
       </c>
       <c r="G89" s="9" t="inlineStr">
@@ -4633,28 +4693,28 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Dịch thuật</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Phân công: nội dung, xử lý đơn, đổi trả/hoàn tiền, hỗ trợ khách</t>
+          <t>Chốt quy ước tên riêng khi dịch (giấy dó, Đông Hồ, Mây)</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr"/>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§12</t>
         </is>
       </c>
       <c r="G90" s="9" t="inlineStr">
@@ -4671,28 +4731,32 @@
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Quyết định nghiệp vụ</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Tham dự buổi đào tạo /admin</t>
-        </is>
-      </c>
-      <c r="D91" s="8" t="inlineStr"/>
+          <t>Q-41: cho phép mua không cần tài khoản (guest checkout)?</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Thay đổi lớn — cần quyết rõ</t>
+        </is>
+      </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§13</t>
         </is>
       </c>
       <c r="G91" s="9" t="inlineStr">
@@ -4709,32 +4773,28 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>14.4</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Quyết định nghiệp vụ</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>UAT: thử đặt đơn thật đầu-cuối + ký biên bản nghiệm thu</t>
-        </is>
-      </c>
-      <c r="D92" s="8" t="inlineStr">
-        <is>
-          <t>COD + payOS, mua tặng với lời chúc chữ/giọng nói/video, huỷ đơn, đổi trả</t>
-        </is>
-      </c>
+          <t>Q-35: đăng ký email đã tồn tại báo "đã đăng ký" hay "kiểm tra email"?</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr"/>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§13</t>
         </is>
       </c>
       <c r="G92" s="9" t="inlineStr">
@@ -4751,28 +4811,32 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>14.5</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Quyết định nghiệp vụ</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Chốt ngày go-live + người quyết định "đạt"</t>
-        </is>
-      </c>
-      <c r="D93" s="8" t="inlineStr"/>
+          <t>Q-21, Q-23, Q-38 và KPI mong muốn</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu giao không in giá; testimonial; ngưỡng chống spam; KPI</t>
+        </is>
+      </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§13</t>
         </is>
       </c>
       <c r="G93" s="9" t="inlineStr">
@@ -4786,9 +4850,203 @@
       <c r="K93" s="9" t="n"/>
       <c r="L93" s="9" t="n"/>
     </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Gửi danh sách người dùng admin (email, vai trò admin/IT)</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr"/>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>🔴 Chặn go-live</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G94" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H94" s="9" t="n"/>
+      <c r="I94" s="10" t="n"/>
+      <c r="J94" s="10" t="n"/>
+      <c r="K94" s="9" t="n"/>
+      <c r="L94" s="9" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Phân công: nội dung, xử lý đơn, đổi trả/hoàn tiền, hỗ trợ khách</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr"/>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>🔴 Chặn go-live</t>
+        </is>
+      </c>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G95" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H95" s="9" t="n"/>
+      <c r="I95" s="10" t="n"/>
+      <c r="J95" s="10" t="n"/>
+      <c r="K95" s="9" t="n"/>
+      <c r="L95" s="9" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Tham dự buổi đào tạo /admin</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr"/>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>🟠 Trước khi mở bán</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G96" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H96" s="9" t="n"/>
+      <c r="I96" s="10" t="n"/>
+      <c r="J96" s="10" t="n"/>
+      <c r="K96" s="9" t="n"/>
+      <c r="L96" s="9" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>UAT: thử đặt đơn thật đầu-cuối + ký biên bản nghiệm thu</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>COD + payOS, mua tặng với lời chúc chữ/giọng nói/video, huỷ đơn, đổi trả</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>🔴 Chặn go-live</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G97" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H97" s="9" t="n"/>
+      <c r="I97" s="10" t="n"/>
+      <c r="J97" s="10" t="n"/>
+      <c r="K97" s="9" t="n"/>
+      <c r="L97" s="9" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>14.5</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Chốt ngày go-live + người quyết định "đạt"</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr"/>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>🟠 Trước khi mở bán</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G98" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H98" s="9" t="n"/>
+      <c r="I98" s="10" t="n"/>
+      <c r="J98" s="10" t="n"/>
+      <c r="K98" s="9" t="n"/>
+      <c r="L98" s="9" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L93"/>
-  <conditionalFormatting sqref="G2:G93">
+  <autoFilter ref="A1:L98"/>
+  <conditionalFormatting sqref="G2:G98">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Xong"</formula>
     </cfRule>
@@ -4802,16 +5060,16 @@
       <formula>"Bị chặn"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I93">
+  <conditionalFormatting sqref="I2:I98">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>AND($I2&lt;&gt;"",$I2&lt;TODAY(),$G2&lt;&gt;"Xong")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chưa bắt đầu,Đang làm,Chờ duyệt,Bị chặn,Xong"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:J93" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nhập ngày dạng dd/mm/yyyy" type="date" operator="greaterThan">
+    <dataValidation sqref="I2:J98" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nhập ngày dạng dd/mm/yyyy" type="date" operator="greaterThan">
       <formula1>36526</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: trang kể chuyện theo từng mẫu đèn (G-108, D-105) + logo fanpage làm favicon
</commit_message>
<xml_diff>
--- a/docs/client-checklist/LAMVI-task-tracker-client.xlsx
+++ b/docs/client-checklist/LAMVI-task-tracker-client.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task tracker" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Task tracker'!$A$1:$L$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Task tracker'!$A$1:$L$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTA('Task tracker'!A2:A98)</f>
+        <f>COUNTA('Task tracker'!A2:A102)</f>
         <v/>
       </c>
     </row>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIF('Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIFS('Task tracker'!E2:E98,"🔴 Chặn go-live",'Task tracker'!G2:G98,"&lt;&gt;Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E102,"🔴 Chặn go-live",'Task tracker'!G2:G102,"&lt;&gt;Xong")</f>
         <v/>
       </c>
     </row>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>SUMPRODUCT(('Task tracker'!I2:I98&lt;&gt;"")*('Task tracker'!I2:I98&lt;TODAY())*('Task tracker'!G2:G98&lt;&gt;"Xong"))</f>
+        <f>SUMPRODUCT(('Task tracker'!I2:I102&lt;&gt;"")*('Task tracker'!I2:I102&lt;TODAY())*('Task tracker'!G2:G102&lt;&gt;"Xong"))</f>
         <v/>
       </c>
     </row>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF('Task tracker'!G2:G98,A11)</f>
+        <f>COUNTIF('Task tracker'!G2:G102,A11)</f>
         <v/>
       </c>
     </row>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF('Task tracker'!G2:G98,A12)</f>
+        <f>COUNTIF('Task tracker'!G2:G102,A12)</f>
         <v/>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF('Task tracker'!G2:G98,A13)</f>
+        <f>COUNTIF('Task tracker'!G2:G102,A13)</f>
         <v/>
       </c>
     </row>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIF('Task tracker'!G2:G98,A14)</f>
+        <f>COUNTIF('Task tracker'!G2:G102,A14)</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIF('Task tracker'!G2:G98,A15)</f>
+        <f>COUNTIF('Task tracker'!G2:G102,A15)</f>
         <v/>
       </c>
     </row>
@@ -690,11 +690,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF('Task tracker'!E2:E98,A18)</f>
+        <f>COUNTIF('Task tracker'!E2:E102,A18)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS('Task tracker'!E2:E98,A18,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E102,A18,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -705,11 +705,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF('Task tracker'!E2:E98,A19)</f>
+        <f>COUNTIF('Task tracker'!E2:E102,A19)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS('Task tracker'!E2:E98,A19,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E102,A19,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -720,11 +720,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIF('Task tracker'!E2:E98,A20)</f>
+        <f>COUNTIF('Task tracker'!E2:E102,A20)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS('Task tracker'!E2:E98,A20,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!E2:E102,A20,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
     </row>
@@ -757,11 +757,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Task tracker'!B2:B98,A24)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A24)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS('Task tracker'!B2:B98,A24,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A24,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D24">
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIF('Task tracker'!B2:B98,A25)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A25)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS('Task tracker'!B2:B98,A25,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A25,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D25">
@@ -795,11 +795,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIF('Task tracker'!B2:B98,A26)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A26)</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS('Task tracker'!B2:B98,A26,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A26,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D26">
@@ -814,11 +814,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIF('Task tracker'!B2:B98,A27)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A27)</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS('Task tracker'!B2:B98,A27,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A27,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D27">
@@ -833,11 +833,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIF('Task tracker'!B2:B98,A28)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A28)</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS('Task tracker'!B2:B98,A28,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A28,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D28">
@@ -852,11 +852,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIF('Task tracker'!B2:B98,A29)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A29)</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS('Task tracker'!B2:B98,A29,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A29,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D29">
@@ -871,11 +871,11 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIF('Task tracker'!B2:B98,A30)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A30)</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS('Task tracker'!B2:B98,A30,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A30,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D30">
@@ -890,11 +890,11 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIF('Task tracker'!B2:B98,A31)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A31)</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS('Task tracker'!B2:B98,A31,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A31,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D31">
@@ -909,11 +909,11 @@
         </is>
       </c>
       <c r="B32">
-        <f>COUNTIF('Task tracker'!B2:B98,A32)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A32)</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS('Task tracker'!B2:B98,A32,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A32,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D32">
@@ -928,11 +928,11 @@
         </is>
       </c>
       <c r="B33">
-        <f>COUNTIF('Task tracker'!B2:B98,A33)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A33)</f>
         <v/>
       </c>
       <c r="C33">
-        <f>COUNTIFS('Task tracker'!B2:B98,A33,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A33,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D33">
@@ -947,11 +947,11 @@
         </is>
       </c>
       <c r="B34">
-        <f>COUNTIF('Task tracker'!B2:B98,A34)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A34)</f>
         <v/>
       </c>
       <c r="C34">
-        <f>COUNTIFS('Task tracker'!B2:B98,A34,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A34,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D34">
@@ -966,11 +966,11 @@
         </is>
       </c>
       <c r="B35">
-        <f>COUNTIF('Task tracker'!B2:B98,A35)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A35)</f>
         <v/>
       </c>
       <c r="C35">
-        <f>COUNTIFS('Task tracker'!B2:B98,A35,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A35,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D35">
@@ -985,11 +985,11 @@
         </is>
       </c>
       <c r="B36">
-        <f>COUNTIF('Task tracker'!B2:B98,A36)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A36)</f>
         <v/>
       </c>
       <c r="C36">
-        <f>COUNTIFS('Task tracker'!B2:B98,A36,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A36,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D36">
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="B37">
-        <f>COUNTIF('Task tracker'!B2:B98,A37)</f>
+        <f>COUNTIF('Task tracker'!B2:B102,A37)</f>
         <v/>
       </c>
       <c r="C37">
-        <f>COUNTIFS('Task tracker'!B2:B98,A37,'Task tracker'!G2:G98,"Xong")</f>
+        <f>COUNTIFS('Task tracker'!B2:B102,A37,'Task tracker'!G2:G102,"Xong")</f>
         <v/>
       </c>
       <c r="D37">
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>32×32, 180×180 (iOS), 512×512. Hiện đang là logo mặc định của Vite</t>
+          <t>32×32, 180×180 (iOS), 512×512. 14/10: đã dùng logo đại diện fanpage (200px) làm favicon 64px + apple-touch-icon; cần file gốc để làm bản 512px</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
@@ -1181,14 +1181,18 @@
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="10" t="n"/>
       <c r="J3" s="10" t="n"/>
       <c r="K3" s="9" t="n"/>
-      <c r="L3" s="9" t="n"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>14/10: đã thay logo Vite bằng logo đại diện fanpage (200px). Cần bản gốc độ phân giải cao</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -1513,22 +1517,22 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Sản phẩm</t>
+          <t>Thương hiệu</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Điền bảng sản phẩm</t>
+          <t>Quyết định thay logo trên thanh menu bằng logo thật (nâu–vàng)</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Tab "Sản phẩm (chữ)" + "Sản phẩm (giá, thông số)" trong file nội dung: tên, mô tả, giá đã gồm VAT, tồn kho</t>
+          <t>Logo fanpage dạng vòng tròn "LV LAMVI" + wordmark có ngọn lửa; web đang dùng chữ triện đỏ dev vẽ tạm. Cần file vector</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1538,28 +1542,24 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>§2</t>
+          <t>§1</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Chờ duyệt</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
       <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="inlineStr">
-        <is>
-          <t>13/10: 5 đèn thật đã lên web (tên, mô tả, thông số, giá tạm). Duyệt tab "Sản phẩm" trong file nội dung</t>
-        </is>
-      </c>
+      <c r="L12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -1569,12 +1569,12 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Điền 6 thông số mỗi đèn</t>
+          <t>Điền bảng sản phẩm</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Kích thước · Chất liệu · Nguồn sáng · Cân nặng · Thời gian làm · Bảo quản</t>
+          <t>Tab "Sản phẩm (chữ)" + "Sản phẩm (giá, thông số)" trong file nội dung: tên, mô tả, giá đã gồm VAT, tồn kho</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1598,14 +1598,14 @@
       <c r="K13" s="9" t="n"/>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>13/10: đã điền 4/6 thông số (kích thước, chất liệu, nguồn sáng, thời gian làm). Thiếu cân nặng, bảo quản → xem 2.7</t>
+          <t>13/10: 5 đèn thật đã lên web (tên, mô tả, thông số, giá tạm). Duyệt tab "Sản phẩm" trong file nội dung</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -1615,12 +1615,12 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Chụp &amp; gửi ảnh sản phẩm thật</t>
+          <t>Điền 6 thông số mỗi đèn</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Vuông ≥1200×1200; đèn bật + tắt; ảnh bối cảnh + chi tiết; kèm alt text tiếng Việt và quyền sử dụng ảnh</t>
+          <t>Kích thước · Chất liệu · Nguồn sáng · Cân nặng · Thời gian làm · Bảo quản</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1635,19 +1635,23 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="10" t="n"/>
       <c r="J14" s="10" t="n"/>
       <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã điền 4/6 thông số (kích thước, chất liệu, nguồn sáng, thời gian làm). Thiếu cân nặng, bảo quản → xem 2.7</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -1657,10 +1661,14 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Chốt bộ Sum Vầy gồm đèn nào, giá lẻ từng đèn (Q-05)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr"/>
+          <t>Chụp &amp; gửi ảnh sản phẩm thật</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Vuông ≥1200×1200; đèn bật + tắt; ảnh bối cảnh + chi tiết; kèm alt text tiếng Việt và quyền sử dụng ảnh</t>
+        </is>
+      </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -1673,23 +1681,19 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Xong</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="10" t="n"/>
       <c r="J15" s="10" t="n"/>
       <c r="K15" s="9" t="n"/>
-      <c r="L15" s="9" t="inlineStr">
-        <is>
-          <t>Không còn áp dụng: không có bộ Sum Vầy (D-104)</t>
-        </is>
-      </c>
+      <c r="L15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -1699,7 +1703,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Chốt có bán sẵn hay làm theo đơn, số tồn ban đầu</t>
+          <t>Chốt bộ Sum Vầy gồm đèn nào, giá lẻ từng đèn (Q-05)</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr"/>
@@ -1715,19 +1719,23 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="10" t="n"/>
       <c r="J16" s="10" t="n"/>
       <c r="K16" s="9" t="n"/>
-      <c r="L16" s="9" t="n"/>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>Không còn áp dụng: không có bộ Sum Vầy (D-104)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -1737,14 +1745,10 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Chốt giá thật từng mẫu trong 5 đèn</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Hiện đang là giá tạm 1.400.000đ cho cả 5 (trung điểm 1,3–1,5 triệu của báo cáo, chưa kiểm chứng)</t>
-        </is>
-      </c>
+          <t>Chốt có bán sẵn hay làm theo đơn, số tồn ban đầu</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr"/>
       <c r="E17" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -1769,7 +1773,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -1779,12 +1783,12 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Gửi cân nặng và cách bảo quản của đèn</t>
+          <t>Chốt giá thật từng mẫu trong 5 đèn</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Hai trong 6 thông số còn trống; xác nhận kích thước chốt (báo cáo ghi 12×12×20 cm là prototype)</t>
+          <t>Hiện đang là giá tạm 1.400.000đ cho cả 5 (trung điểm 1,3–1,5 triệu của báo cáo, chưa kiểm chứng)</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1811,7 +1815,7 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -1821,17 +1825,17 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Viết mô tả dài / câu chuyện cho từng đèn</t>
+          <t>Gửi cân nặng và cách bảo quản của đèn</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Content Plan đã có bài dài cho 5 đèn; web hiện chỉ có mô tả 1 câu — cho biết dùng nguyên bài hay rút gọn</t>
+          <t>Hai trong 6 thông số còn trống; xác nhận kích thước chốt (báo cáo ghi 12×12×20 cm là prototype)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1853,53 +1857,49 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Bộ sưu tập</t>
+          <t>Sản phẩm</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Điền nội dung mỗi bộ sưu tập</t>
+          <t>Viết mô tả dài / câu chuyện cho từng đèn</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Tab "Bộ sưu tập": tên, mô tả, câu chuyện; ảnh bìa ngang ≥1600px</t>
+          <t>Content Plan đã có bài dài cho 5 đèn; web hiện chỉ có mô tả 1 câu — cho biết dùng nguyên bài hay rút gọn</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>§3</t>
+          <t>§2</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Chờ duyệt</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="10" t="n"/>
       <c r="J20" s="10" t="n"/>
       <c r="K20" s="9" t="n"/>
-      <c r="L20" s="9" t="inlineStr">
-        <is>
-          <t>13/10: 1 bộ "Bộ sưu tập đầu tiên" + câu chuyện bộ do dev soạn từ Content Plan</t>
-        </is>
-      </c>
+      <c r="L20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -1909,17 +1909,17 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Chốt có thêm category/bộ lọc khác không</t>
+          <t>Điền nội dung mỗi bộ sưu tập</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Theo dịp (Tết, Trung thu, tân gia…), theo không gian (bàn trà, phòng ngủ…), theo giá</t>
+          <t>Tab "Bộ sưu tập": tên, mô tả, câu chuyện; ảnh bìa ngang ≥1600px</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1929,19 +1929,23 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H21" s="9" t="n"/>
       <c r="I21" s="10" t="n"/>
       <c r="J21" s="10" t="n"/>
       <c r="K21" s="9" t="n"/>
-      <c r="L21" s="9" t="n"/>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>13/10: 1 bộ "Bộ sưu tập đầu tiên" + câu chuyện bộ do dev soạn từ Content Plan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -1951,12 +1955,12 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Viết nội dung phần thưởng cốt truyện cho Gallery / chăn Đông Hồ</t>
+          <t>Chốt có thêm category/bộ lọc khác không</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Và xác nhận còn muốn giữ tính năng này</t>
+          <t>Theo dịp (Tết, Trung thu, tân gia…), theo không gian (bàn trà, phòng ngủ…), theo giá</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1983,32 +1987,32 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Trang chủ</t>
+          <t>Bộ sưu tập</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Duyệt/sửa Hero (HOME-02) + gửi ảnh hoặc video hero thật</t>
+          <t>Viết nội dung phần thưởng cốt truyện cho Gallery / chăn Đông Hồ</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận "làng nghề trăm năm" đúng sự thật</t>
+          <t>Và xác nhận còn muốn giữ tính năng này</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>§4</t>
+          <t>§3</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -2025,7 +2029,7 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -2035,13 +2039,17 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Duyệt dải chữ chạy (HOME-03)</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr"/>
+          <t>Duyệt/sửa Hero (HOME-02) + gửi ảnh hoặc video hero thật</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Xác nhận "làng nghề trăm năm" đúng sự thật</t>
+        </is>
+      </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -2063,7 +2071,7 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -2073,17 +2081,13 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Gửi số liệu thật + câu chuyện làng nghề (HOME-04)</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>79+ năm, 10 nghệ nhân hiện là số MẪU</t>
-        </is>
-      </c>
+          <t>Duyệt dải chữ chạy (HOME-03)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -2093,23 +2097,19 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Chờ duyệt</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="10" t="n"/>
       <c r="J25" s="10" t="n"/>
       <c r="K25" s="9" t="n"/>
-      <c r="L25" s="9" t="inlineStr">
-        <is>
-          <t>13/10: đã thay số mẫu bằng 5 đèn / 3 chặng / 1 lời chúc. Cần câu chuyện làng nghề thật</t>
-        </is>
-      </c>
+      <c r="L25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Khối Nghệ nhân (HOME-05): gửi nhân vật thật hoặc bỏ khối</t>
+          <t>Gửi số liệu thật + câu chuyện làng nghề (HOME-04)</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Tên, ảnh chân dung, câu nói, 32 năm / 4.000+ đèn là mẫu; cần văn bản đồng ý của nghệ nhân</t>
+          <t>79+ năm, 10 nghệ nhân hiện là số MẪU</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -2148,14 +2148,14 @@
       <c r="K26" s="9" t="n"/>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>13/10: đã dùng tên Nghệ nhân Ưu tú Nguyễn Hữu Quả, bỏ câu trích + số liệu mẫu. Cần ảnh + đồng ý → xem 8.11</t>
+          <t>13/10: đã thay số mẫu bằng 5 đèn / 3 chặng / 1 lời chúc. Cần câu chuyện làng nghề thật</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -2165,13 +2165,17 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Duyệt câu giới thiệu bộ sưu tập (HOME-06)</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr"/>
+          <t>Khối Nghệ nhân (HOME-05): gửi nhân vật thật hoặc bỏ khối</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Tên, ảnh chân dung, câu nói, 32 năm / 4.000+ đèn là mẫu; cần văn bản đồng ý của nghệ nhân</t>
+        </is>
+      </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -2181,19 +2185,23 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="10" t="n"/>
       <c r="J27" s="10" t="n"/>
       <c r="K27" s="9" t="n"/>
-      <c r="L27" s="9" t="n"/>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã dùng tên Nghệ nhân Ưu tú Nguyễn Hữu Quả, bỏ câu trích + số liệu mẫu. Cần ảnh + đồng ý → xem 8.11</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
@@ -2203,7 +2211,7 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Lookbook (HOME-07): gửi ảnh thật + chốt 5 tên màu</t>
+          <t>Duyệt câu giới thiệu bộ sưu tập (HOME-06)</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr"/>
@@ -2219,23 +2227,19 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Chờ duyệt</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="10" t="n"/>
       <c r="J28" s="10" t="n"/>
       <c r="K28" s="9" t="n"/>
-      <c r="L28" s="9" t="inlineStr">
-        <is>
-          <t>13/10: lookbook = 5 tên đèn. Cần ảnh thật</t>
-        </is>
-      </c>
+      <c r="L28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -2245,7 +2249,7 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Hành trình thủ công (HOME-08): xác nhận 4 bước + ảnh/video từng bước</t>
+          <t>Lookbook (HOME-07): gửi ảnh thật + chốt 5 tên màu</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr"/>
@@ -2270,14 +2274,14 @@
       <c r="K29" s="9" t="n"/>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>13/10: 4 bước đã đổi theo Content Plan. Cần xác nhận + ảnh/video</t>
+          <t>13/10: lookbook = 5 tên đèn. Cần ảnh thật</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
@@ -2287,14 +2291,10 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Duyệt khối Trải nghiệm QR (HOME-09)</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Nhất là câu thời hạn lưu 30 ngày</t>
-        </is>
-      </c>
+          <t>Hành trình thủ công (HOME-08): xác nhận 4 bước + ảnh/video từng bước</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr"/>
       <c r="E30" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2316,14 +2316,14 @@
       <c r="K30" s="9" t="n"/>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>13/10: đã sửa QR chỉ ở thiệp cảm ơn (D-104)</t>
+          <t>13/10: 4 bước đã đổi theo Content Plan. Cần xác nhận + ảnh/video</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -2333,17 +2333,17 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Testimonials (HOME-10): gửi đánh giá thật + đồng ý của người viết, hoặc bỏ</t>
+          <t>Duyệt khối Trải nghiệm QR (HOME-09)</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Hiện đang ẩn</t>
+          <t>Nhất là câu thời hạn lưu 30 ngày</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -2353,19 +2353,23 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H31" s="9" t="n"/>
       <c r="I31" s="10" t="n"/>
       <c r="J31" s="10" t="n"/>
       <c r="K31" s="9" t="n"/>
-      <c r="L31" s="9" t="n"/>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>13/10: đã sửa QR chỉ ở thiệp cảm ơn (D-104)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
@@ -2375,17 +2379,17 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Duyệt 5 FAQ + thêm câu hỏi thực tế khách hay hỏi (HOME-11)</t>
+          <t>Testimonials (HOME-10): gửi đánh giá thật + đồng ý của người viết, hoặc bỏ</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Tab "FAQ"</t>
+          <t>Hiện đang ẩn</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -2395,23 +2399,19 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Chờ duyệt</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="10" t="n"/>
       <c r="J32" s="10" t="n"/>
       <c r="K32" s="9" t="n"/>
-      <c r="L32" s="9" t="inlineStr">
-        <is>
-          <t>13/10: FAQ 9 câu (thêm 4 câu). Cần thêm câu hỏi thực tế</t>
-        </is>
-      </c>
+      <c r="L32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>4.11</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -2421,13 +2421,17 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Duyệt tiêu đề/mô tả SEO hiện trên Google</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr"/>
+          <t>Duyệt 5 FAQ + thêm câu hỏi thực tế khách hay hỏi (HOME-11)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Tab "FAQ"</t>
+        </is>
+      </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -2437,19 +2441,23 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H33" s="9" t="n"/>
       <c r="I33" s="10" t="n"/>
       <c r="J33" s="10" t="n"/>
       <c r="K33" s="9" t="n"/>
-      <c r="L33" s="9" t="n"/>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>13/10: FAQ 9 câu (thêm 4 câu). Cần thêm câu hỏi thực tế</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>4.11</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
@@ -2459,13 +2467,13 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Chốt giữ hay bỏ form newsletter (G-11)</t>
+          <t>Duyệt tiêu đề/mô tả SEO hiện trên Google</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr"/>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -2487,32 +2495,28 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Các trang khác</t>
+          <t>Trang chủ</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Cửa hàng / Chi tiết sản phẩm / Bộ sưu tập</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Tab "Nội dung web"</t>
-        </is>
-      </c>
+          <t>Chốt giữ hay bỏ form newsletter (G-11)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr"/>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>§5</t>
+          <t>§4</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -2529,7 +2533,7 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -2539,10 +2543,14 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Giỏ hàng / Thanh toán / Đơn hàng</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr"/>
+          <t>Duyệt chữ Cửa hàng / Chi tiết sản phẩm / Bộ sưu tập</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Tab "Nội dung web"</t>
+        </is>
+      </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2567,7 +2575,7 @@
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -2577,7 +2585,7 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Đăng nhập / Đăng ký / Quên mật khẩu + gửi ảnh nền thương hiệu</t>
+          <t>Duyệt chữ Giỏ hàng / Thanh toán / Đơn hàng</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr"/>
@@ -2605,7 +2613,7 @@
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
@@ -2615,14 +2623,10 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ trang người nhận mở lời chúc (QR-GIFT)</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Điểm chạm cảm xúc nhất — nên do copywriter viết</t>
-        </is>
-      </c>
+          <t>Duyệt chữ Đăng nhập / Đăng ký / Quên mật khẩu + gửi ảnh nền thương hiệu</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr"/>
       <c r="E38" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2647,7 +2651,7 @@
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -2657,10 +2661,14 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Duyệt chữ Liên hệ, 404, bảo trì</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr"/>
+          <t>Duyệt chữ trang người nhận mở lời chúc (QR-GIFT)</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Điểm chạm cảm xúc nhất — nên do copywriter viết</t>
+        </is>
+      </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2685,7 +2693,7 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
@@ -2695,14 +2703,10 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Duyệt tên các trạng thái đơn hàng</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Chờ thanh toán, Đang làm, Đã đóng gói, Đã gửi, Đã giao, Đã huỷ, Hoàn tiền</t>
-        </is>
-      </c>
+          <t>Duyệt chữ Liên hệ, 404, bảo trì</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr"/>
       <c r="E40" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -2727,22 +2731,22 @@
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Mây (AI)</t>
+          <t>Các trang khác</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Chốt tính cách &amp; giọng nói của Mây</t>
+          <t>Duyệt tên các trạng thái đơn hàng</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Xưng hô, từ nên/cấm dùng, độ dài câu trả lời</t>
+          <t>Chờ thanh toán, Đang làm, Đã đóng gói, Đã gửi, Đã giao, Đã huỷ, Hoàn tiền</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2752,7 +2756,7 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>§6</t>
+          <t>§5</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
@@ -2769,7 +2773,7 @@
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
@@ -2779,17 +2783,17 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Viết kho kiến thức cho Mây (≥30 câu FAQ)</t>
+          <t>Chốt tính cách &amp; giọng nói của Mây</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Chất liệu, quy trình, bảo quản, an toàn, quà doanh nghiệp, in logo…</t>
+          <t>Xưng hô, từ nên/cấm dùng, độ dài câu trả lời</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -2799,23 +2803,19 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="10" t="n"/>
       <c r="J42" s="10" t="n"/>
       <c r="K42" s="9" t="n"/>
-      <c r="L42" s="9" t="inlineStr">
-        <is>
-          <t>13/10: FAQ mới 9 câu — Mây dùng FAQ làm kiến thức</t>
-        </is>
-      </c>
+      <c r="L42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -2825,13 +2825,17 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Danh sách chủ đề Mây không được trả lời / phải chuyển nhân viên</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr"/>
+          <t>Viết kho kiến thức cho Mây (≥30 câu FAQ)</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Chất liệu, quy trình, bảo quản, an toàn, quà doanh nghiệp, in logo…</t>
+        </is>
+      </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -2841,19 +2845,23 @@
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H43" s="9" t="n"/>
       <c r="I43" s="10" t="n"/>
       <c r="J43" s="10" t="n"/>
       <c r="K43" s="9" t="n"/>
-      <c r="L43" s="9" t="n"/>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>13/10: FAQ mới 9 câu — Mây dùng FAQ làm kiến thức</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
@@ -2863,17 +2871,13 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Cung cấp kênh chuyển nhân viên + giờ trực</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Zalo / hotline / email</t>
-        </is>
-      </c>
+          <t>Danh sách chủ đề Mây không được trả lời / phải chuyển nhân viên</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr"/>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -2895,7 +2899,7 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -2905,17 +2909,17 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Duyệt câu báo lỗi, câu gợi ý, câu chào, tour 5 bước</t>
+          <t>Cung cấp kênh chuyển nhân viên + giờ trực</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Tab "Mây" và "Nội dung web"</t>
+          <t>Zalo / hotline / email</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -2925,23 +2929,19 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>Chờ duyệt</t>
+          <t>Chưa bắt đầu</t>
         </is>
       </c>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="10" t="n"/>
       <c r="J45" s="10" t="n"/>
       <c r="K45" s="9" t="n"/>
-      <c r="L45" s="9" t="inlineStr">
-        <is>
-          <t>13/10: câu tour về QR đã sửa theo D-104</t>
-        </is>
-      </c>
+      <c r="L45" s="9" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
@@ -2951,12 +2951,12 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Chốt hạn mức &amp; ngân sách OpenAI</t>
+          <t>Duyệt câu báo lỗi, câu gợi ý, câu chào, tour 5 bước</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Hiện 20 USD/tháng; 20/50/100 tin nhắn</t>
+          <t>Tab "Mây" và "Nội dung web"</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2971,19 +2971,23 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="10" t="n"/>
       <c r="J46" s="10" t="n"/>
       <c r="K46" s="9" t="n"/>
-      <c r="L46" s="9" t="n"/>
+      <c r="L46" s="9" t="inlineStr">
+        <is>
+          <t>13/10: câu tour về QR đã sửa theo D-104</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -2993,13 +2997,17 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Pháp chế duyệt thông báo xử lý dữ liệu ở nước ngoài + quyền xoá lịch sử chat (I-15)</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr"/>
+          <t>Chốt hạn mức &amp; ngân sách OpenAI</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Hiện 20 USD/tháng; 20/50/100 tin nhắn</t>
+        </is>
+      </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -3021,24 +3029,20 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Lô đèn &amp; QR</t>
+          <t>Mây (AI)</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Quay &amp; gửi video quy trình cho lô đầu tiên</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Mã lô, ngày làm, tiêu đề VI/EN/ZH, câu chuyện, file MP4/WebM/MOV ≤500 MB</t>
-        </is>
-      </c>
+          <t>Pháp chế duyệt thông báo xử lý dữ liệu ở nước ngoài + quyền xoá lịch sử chat (I-15)</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr"/>
       <c r="E48" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3046,7 +3050,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>§7</t>
+          <t>§6</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
@@ -3063,7 +3067,7 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -3073,13 +3077,17 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Chốt quy tắc đặt mã lô + quy trình in thiệp có QR (không khắc lên đèn)</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr"/>
+          <t>Quay &amp; gửi video quy trình cho lô đầu tiên</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Mã lô, ngày làm, tiêu đề VI/EN/ZH, câu chuyện, file MP4/WebM/MOV ≤500 MB</t>
+        </is>
+      </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -3101,7 +3109,7 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
@@ -3111,14 +3119,10 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Thiết kế thiệp cảm ơn có mã QR</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Kích thước, mặt trước/sau, mẫu viết tay hay in</t>
-        </is>
-      </c>
+          <t>Chốt quy tắc đặt mã lô + quy trình in thiệp có QR (không khắc lên đèn)</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr"/>
       <c r="E50" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -3143,7 +3147,7 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -3153,13 +3157,17 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận chính sách lưu trữ lời chúc (30 ngày giọng nói/video)</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr"/>
+          <t>Thiết kế thiệp cảm ơn có mã QR</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Kích thước, mặt trước/sau, mẫu viết tay hay in</t>
+        </is>
+      </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -3181,7 +3189,7 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
@@ -3191,22 +3199,18 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Trả lời Q-12, Q-14, Q-25, Q-27, Q-29, Q-33</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Phí thiệp; admin xem lời chúc; QR đơn tự mua; xem trước; lời chúc không phải tiếng Việt; PIN</t>
-        </is>
-      </c>
+          <t>Xác nhận chính sách lưu trữ lời chúc (30 ngày giọng nói/video)</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr"/>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>§7/§13</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -3223,7 +3227,7 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -3233,12 +3237,12 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Quyết định trang kể chuyện theo từng mẫu đèn (QR trên thiệp)</t>
+          <t>Trả lời Q-12, Q-14, Q-25, Q-27, Q-29, Q-33</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Content Plan 30/10: QR mở nội dung riêng của mẫu (artwork, chi tiết) rồi mới tới lời chúc. Web chưa có (G-108) — chốt phạm vi + nội dung</t>
+          <t>Phí thiệp; admin xem lời chúc; QR đơn tự mua; xem trước; lời chúc không phải tiếng Việt; PIN</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -3248,7 +3252,7 @@
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>§7</t>
+          <t>§7/§13</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
@@ -3265,96 +3269,116 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Gửi tên pháp nhân + tên thương mại</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr"/>
+          <t>Trang kể chuyện theo từng mẫu đèn (QR trên thiệp)</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Content Plan 30/10: QR mở câu chuyện của mẫu rồi mới tới lời chúc (G-108, D-105)</t>
+        </is>
+      </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="10" t="n"/>
       <c r="J54" s="10" t="n"/>
       <c r="K54" s="9" t="n"/>
-      <c r="L54" s="9" t="n"/>
+      <c r="L54" s="9" t="inlineStr">
+        <is>
+          <t>14/10: đã làm trang kể chuyện theo mẫu đèn (D-105): QR thiệp → câu chuyện → lời chúc; tab Câu chuyện ở trang sản phẩm</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>7.7</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Gửi MST / số ĐKKD, ngày cấp, nơi cấp</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr"/>
+          <t>Duyệt câu chuyện 5 đèn (VI/EN/ZH)</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Tab "Câu chuyện" ở trang sản phẩm + trang lời chúc. Sửa ở /admin → Sản phẩm → Câu chuyện của mẫu đèn, hoặc tab "Sản phẩm (chữ)" trong file nội dung</t>
+        </is>
+      </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="10" t="n"/>
       <c r="J55" s="10" t="n"/>
       <c r="K55" s="9" t="n"/>
-      <c r="L55" s="9" t="n"/>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>14/10: 5 câu chuyện vi/en/zh đã lên web, soạn từ Content Plan + 2 bài của nhóm</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Gửi địa chỉ trụ sở + địa chỉ xưởng</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr"/>
+          <t>Gửi ảnh gốc từng mẫu đèn (đèn bật/tắt, cận cảnh)</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Poster trên fanpage chỉ lấy được ≤206 px khi chưa đăng nhập. Sản phẩm thật là đèn TRỤ trên đế gỗ tối màu; hình minh hoạ trên web đang là lồng đèn → cần thay bằng ảnh thật</t>
+        </is>
+      </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3362,7 +3386,7 @@
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
@@ -3379,20 +3403,24 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Doanh nghiệp &amp; pháp lý</t>
+          <t>Lô đèn &amp; QR</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Gửi hotline, Zalo, email hỗ trợ, giờ làm việc</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr"/>
+          <t>Xác nhận thông tin liên hệ trên banner fanpage</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Địa chỉ Làng Khánh S – Vinhomes Thăng Long; hotline 0962 254 128; email lamvi6866@ (banner) vs lamvi6886@ (mục Giới thiệu); website lamvi.com.vn; TikTok @lamvi360 (G-115)</t>
+        </is>
+      </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3400,7 +3428,7 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>§8</t>
+          <t>§7/§8</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
@@ -3417,7 +3445,7 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
@@ -3427,17 +3455,13 @@
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Gửi link mạng xã hội</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Facebook, Instagram, TikTok, Zalo OA, YouTube (https)</t>
-        </is>
-      </c>
+          <t>Gửi tên pháp nhân + tên thương mại</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr"/>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -3459,7 +3483,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>8.6</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -3469,14 +3493,10 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Thông báo website TMĐT với Bộ Công Thương + gửi link xác nhận</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>online.gov.vn (Q-42)</t>
-        </is>
-      </c>
+          <t>Gửi MST / số ĐKKD, ngày cấp, nơi cấp</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr"/>
       <c r="E59" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3501,7 +3521,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
@@ -3511,14 +3531,10 @@
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Chỉ định người đại diện / bên kiểm soát dữ liệu + email nhận yêu cầu dữ liệu</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>Q-40</t>
-        </is>
-      </c>
+          <t>Gửi địa chỉ trụ sở + địa chỉ xưởng</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr"/>
       <c r="E60" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3543,7 +3559,7 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -3553,7 +3569,7 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Chốt tên miền chính thức + cấp quyền DNS</t>
+          <t>Gửi hotline, Zalo, email hỗ trợ, giờ làm việc</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr"/>
@@ -3581,7 +3597,7 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
@@ -3591,17 +3607,17 @@
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Pháp chế duyệt 5 trang chính sách + banner cookie/GA</t>
+          <t>Gửi link mạng xã hội</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>Q-40, Q-42, Q-43</t>
+          <t>Facebook, Instagram, TikTok, Zalo OA, YouTube (https)</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -3623,7 +3639,7 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>8.10</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -3633,10 +3649,14 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>Giấy phép ảnh: tư liệu Đông Hồ (Q-36), ảnh nghệ nhân, ảnh sản phẩm</t>
-        </is>
-      </c>
-      <c r="D63" s="8" t="inlineStr"/>
+          <t>Thông báo website TMĐT với Bộ Công Thương + gửi link xác nhận</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>online.gov.vn (Q-42)</t>
+        </is>
+      </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3661,7 +3681,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
@@ -3671,12 +3691,12 @@
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Gửi ảnh chân dung + văn bản đồng ý của Nghệ nhân Ưu tú Nguyễn Hữu Quả</t>
+          <t>Chỉ định người đại diện / bên kiểm soát dữ liệu + email nhận yêu cầu dữ liệu</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>Web đã dùng tên thật theo Content Plan; ảnh vẫn là hình minh hoạ. Không đưa phần "Tài liệu tham khảo" trích nguồn ngoài lên web khi chưa xin phép</t>
+          <t>Q-40</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -3686,7 +3706,7 @@
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>§4/§8</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
@@ -3703,24 +3723,20 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Chốt phí ship + ngưỡng freeship</t>
-        </is>
-      </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Hiện 30.000đ, miễn phí từ 1.000.000đ (giả định)</t>
-        </is>
-      </c>
+          <t>Chốt tên miền chính thức + cấp quyền DNS</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr"/>
       <c r="E65" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3728,7 +3744,7 @@
       </c>
       <c r="F65" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
@@ -3745,20 +3761,24 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Chốt đơn vị vận chuyển, thời gian giao theo vùng, vùng không giao</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="inlineStr"/>
+          <t>Pháp chế duyệt 5 trang chính sách + banner cookie/GA</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Q-40, Q-42, Q-43</t>
+        </is>
+      </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3766,7 +3786,7 @@
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G66" s="9" t="inlineStr">
@@ -3783,17 +3803,17 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>8.10</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận thời gian làm đèn (5–7 ngày làm việc?)</t>
+          <t>Giấy phép ảnh: tư liệu Đông Hồ (Q-36), ảnh nghệ nhân, ảnh sản phẩm</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr"/>
@@ -3804,7 +3824,7 @@
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§8</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
@@ -3821,22 +3841,22 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Vận hành bán hàng</t>
+          <t>Doanh nghiệp &amp; pháp lý</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Xác nhận VAT 10% + cách xuất hoá đơn điện tử</t>
+          <t>Gửi ảnh chân dung + văn bản đồng ý của Nghệ nhân Ưu tú Nguyễn Hữu Quả</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Hệ thống chưa có xuất hoá đơn</t>
+          <t>Web đã dùng tên thật theo Content Plan; ảnh vẫn là hình minh hoạ. Không đưa phần "Tài liệu tham khảo" trích nguồn ngoài lên web khi chưa xin phép</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -3846,7 +3866,7 @@
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>§9</t>
+          <t>§4/§8</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
@@ -3863,7 +3883,7 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
@@ -3873,10 +3893,14 @@
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Mở tài khoản payOS + quyết định COD (giới hạn giá trị? Q-37)</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr"/>
+          <t>Chốt phí ship + ngưỡng freeship</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Hiện 30.000đ, miễn phí từ 1.000.000đ (giả định)</t>
+        </is>
+      </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -3901,7 +3925,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
@@ -3911,17 +3935,13 @@
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Chốt chính sách đổi trả còn mở</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>Q-06 trả 1 đèn trong bộ; Q-20 mức hoàn khi huỷ đơn đã thanh toán; thời gian hoàn tiền; ai chịu phí ship đổi trả</t>
-        </is>
-      </c>
+          <t>Chốt đơn vị vận chuyển, thời gian giao theo vùng, vùng không giao</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr"/>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -3943,7 +3963,7 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
@@ -3953,13 +3973,13 @@
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Lên danh sách coupon ra mắt</t>
+          <t>Xác nhận thời gian làm đèn (5–7 ngày làm việc?)</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr"/>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -3981,7 +4001,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
@@ -3991,13 +4011,17 @@
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Chốt có bán quà doanh nghiệp / in logo không</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr"/>
+          <t>Xác nhận VAT 10% + cách xuất hoá đơn điện tử</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Hệ thống chưa có xuất hoá đơn</t>
+        </is>
+      </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -4019,7 +4043,7 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
@@ -4029,13 +4053,13 @@
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Mô tả quy trình xử lý đơn nội bộ (ai làm gì, khi nào đổi trạng thái)</t>
+          <t>Mở tài khoản payOS + quyết định COD (giới hạn giá trị? Q-37)</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr"/>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -4057,7 +4081,7 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>9.10</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
@@ -4067,13 +4091,17 @@
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Chốt chính sách bảo hành (nếu có)</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr"/>
+          <t>Chốt chính sách đổi trả còn mở</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Q-06 trả 1 đèn trong bộ; Q-20 mức hoàn khi huỷ đơn đã thanh toán; thời gian hoàn tiền; ai chịu phí ship đổi trả</t>
+        </is>
+      </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -4095,24 +4123,20 @@
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Duyệt nội dung email giao dịch</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>Tab "Email"</t>
-        </is>
-      </c>
+          <t>Lên danh sách coupon ra mắt</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr"/>
       <c r="E75" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -4120,7 +4144,7 @@
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>§10</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
@@ -4137,32 +4161,28 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Chọn địa chỉ gửi + xác minh tên miền gửi (SPF/DKIM)</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Cần quyền DNS</t>
-        </is>
-      </c>
+          <t>Chốt có bán quà doanh nghiệp / in logo không</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr"/>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>§10</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G76" s="9" t="inlineStr">
@@ -4179,28 +4199,28 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Chốt có SMS/Zalo thông báo đơn không (Q-24)</t>
+          <t>Mô tả quy trình xử lý đơn nội bộ (ai làm gì, khi nào đổi trạng thái)</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr"/>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>§10</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
@@ -4217,28 +4237,28 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>9.10</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Vận hành bán hàng</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Tên miền + DNS</t>
+          <t>Chốt chính sách bảo hành (nếu có)</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr"/>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§9</t>
         </is>
       </c>
       <c r="G78" s="9" t="inlineStr">
@@ -4255,28 +4275,32 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Tạo / cấp quyền Vercel</t>
-        </is>
-      </c>
-      <c r="D79" s="8" t="inlineStr"/>
+          <t>Duyệt nội dung email giao dịch</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Tab "Email"</t>
+        </is>
+      </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§10</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
@@ -4293,20 +4317,24 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Tạo project Supabase production (gói phù hợp, có sao lưu)</t>
-        </is>
-      </c>
-      <c r="D80" s="8" t="inlineStr"/>
+          <t>Chọn địa chỉ gửi + xác minh tên miền gửi (SPF/DKIM)</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Cần quyền DNS</t>
+        </is>
+      </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -4314,7 +4342,7 @@
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§10</t>
         </is>
       </c>
       <c r="G80" s="9" t="inlineStr">
@@ -4331,32 +4359,28 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản dịch vụ</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Đăng ký payOS, lấy Client ID / API Key / Checksum Key</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr">
-        <is>
-          <t>Chia sẻ khoá qua kênh an toàn</t>
-        </is>
-      </c>
+          <t>Chốt có SMS/Zalo thông báo đơn không (Q-24)</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr"/>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>§11</t>
+          <t>§10</t>
         </is>
       </c>
       <c r="G81" s="9" t="inlineStr">
@@ -4373,7 +4397,7 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
@@ -4383,7 +4407,7 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Resend hoặc Brevo</t>
+          <t>Tên miền + DNS</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr"/>
@@ -4411,7 +4435,7 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
@@ -4421,13 +4445,13 @@
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Google Analytics 4: Measurement ID + quyền Viewer</t>
+          <t>Tạo / cấp quyền Vercel</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr"/>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -4449,7 +4473,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
@@ -4459,17 +4483,13 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Google Cloud OAuth (đăng nhập bằng Google)</t>
-        </is>
-      </c>
-      <c r="D84" s="8" t="inlineStr">
-        <is>
-          <t>Cần logo + chính sách riêng tư + miền thật</t>
-        </is>
-      </c>
+          <t>Tạo project Supabase production (gói phù hợp, có sao lưu)</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr"/>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
@@ -4491,7 +4511,7 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
@@ -4501,13 +4521,17 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>OpenAI API key + hạn mức chi tiêu</t>
-        </is>
-      </c>
-      <c r="D85" s="8" t="inlineStr"/>
+          <t>Đăng ký payOS, lấy Client ID / API Key / Checksum Key</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Chia sẻ khoá qua kênh an toàn</t>
+        </is>
+      </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
@@ -4529,7 +4553,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>11.9</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
@@ -4539,13 +4563,13 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Google Search Console (xác minh tên miền)</t>
+          <t>Tài khoản Resend hoặc Brevo</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr"/>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F86" s="8" t="inlineStr">
@@ -4567,7 +4591,7 @@
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>11.10</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
@@ -4577,17 +4601,13 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Quyết định gắn pixel quảng cáo (Facebook/TikTok)</t>
-        </is>
-      </c>
-      <c r="D87" s="8" t="inlineStr">
-        <is>
-          <t>Cần cập nhật banner cookie</t>
-        </is>
-      </c>
+          <t>Google Analytics 4: Measurement ID + quyền Viewer</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr"/>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F87" s="8" t="inlineStr">
@@ -4609,22 +4629,22 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>Dịch thuật</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Chốt có bán cho khách EN / ZH không</t>
+          <t>Google Cloud OAuth (đăng nhập bằng Google)</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>Nếu không thì có thể ẩn để giảm công duy trì</t>
+          <t>Cần logo + chính sách riêng tư + miền thật</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -4634,7 +4654,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G88" s="9" t="inlineStr">
@@ -4651,32 +4671,28 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>11.8</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>Dịch thuật</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Thuê người bản ngữ duyệt bản EN / ZH</t>
-        </is>
-      </c>
-      <c r="D89" s="8" t="inlineStr">
-        <is>
-          <t>Tên sản phẩm, câu chuyện, chính sách, email</t>
-        </is>
-      </c>
+          <t>OpenAI API key + hạn mức chi tiêu</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr"/>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>🟡 Làm sau được</t>
+          <t>🟠 Trước khi mở bán</t>
         </is>
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G89" s="9" t="inlineStr">
@@ -4693,17 +4709,17 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>11.9</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Dịch thuật</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Chốt quy ước tên riêng khi dịch (giấy dó, Đông Hồ, Mây)</t>
+          <t>Google Search Console (xác minh tên miền)</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr"/>
@@ -4714,7 +4730,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>§12</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G90" s="9" t="inlineStr">
@@ -4731,32 +4747,32 @@
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>11.10</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Quyết định nghiệp vụ</t>
+          <t>Tài khoản dịch vụ</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Q-41: cho phép mua không cần tài khoản (guest checkout)?</t>
+          <t>Quyết định gắn pixel quảng cáo (Facebook/TikTok)</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Thay đổi lớn — cần quyết rõ</t>
+          <t>Cần cập nhật banner cookie</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>§13</t>
+          <t>§11</t>
         </is>
       </c>
       <c r="G91" s="9" t="inlineStr">
@@ -4773,20 +4789,24 @@
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>Quyết định nghiệp vụ</t>
+          <t>Dịch thuật</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Q-35: đăng ký email đã tồn tại báo "đã đăng ký" hay "kiểm tra email"?</t>
-        </is>
-      </c>
-      <c r="D92" s="8" t="inlineStr"/>
+          <t>Chốt có bán cho khách EN / ZH không</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Nếu không thì có thể ẩn để giảm công duy trì</t>
+        </is>
+      </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
           <t>🟠 Trước khi mở bán</t>
@@ -4794,7 +4814,7 @@
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>§13</t>
+          <t>§12</t>
         </is>
       </c>
       <c r="G92" s="9" t="inlineStr">
@@ -4811,22 +4831,22 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Quyết định nghiệp vụ</t>
+          <t>Dịch thuật</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Q-21, Q-23, Q-38 và KPI mong muốn</t>
+          <t>Thuê người bản ngữ duyệt bản EN / ZH</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Phiếu giao không in giá; testimonial; ngưỡng chống spam; KPI</t>
+          <t>Tên sản phẩm, câu chuyện, chính sách, email</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -4836,7 +4856,7 @@
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>§13</t>
+          <t>§12</t>
         </is>
       </c>
       <c r="G93" s="9" t="inlineStr">
@@ -4853,28 +4873,28 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Dịch thuật</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>Gửi danh sách người dùng admin (email, vai trò admin/IT)</t>
+          <t>Chốt quy ước tên riêng khi dịch (giấy dó, Đông Hồ, Mây)</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr"/>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§12</t>
         </is>
       </c>
       <c r="G94" s="9" t="inlineStr">
@@ -4891,20 +4911,24 @@
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Quyết định nghiệp vụ</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Phân công: nội dung, xử lý đơn, đổi trả/hoàn tiền, hỗ trợ khách</t>
-        </is>
-      </c>
-      <c r="D95" s="8" t="inlineStr"/>
+          <t>Q-41: cho phép mua không cần tài khoản (guest checkout)?</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Thay đổi lớn — cần quyết rõ</t>
+        </is>
+      </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
           <t>🔴 Chặn go-live</t>
@@ -4912,7 +4936,7 @@
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§13</t>
         </is>
       </c>
       <c r="G95" s="9" t="inlineStr">
@@ -4929,17 +4953,17 @@
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Quyết định nghiệp vụ</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>Tham dự buổi đào tạo /admin</t>
+          <t>Q-35: đăng ký email đã tồn tại báo "đã đăng ký" hay "kiểm tra email"?</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr"/>
@@ -4950,7 +4974,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§13</t>
         </is>
       </c>
       <c r="G96" s="9" t="inlineStr">
@@ -4967,32 +4991,32 @@
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>14.4</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Admin &amp; vận hành</t>
+          <t>Quyết định nghiệp vụ</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>UAT: thử đặt đơn thật đầu-cuối + ký biên bản nghiệm thu</t>
+          <t>Q-21, Q-23, Q-38 và KPI mong muốn</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>COD + payOS, mua tặng với lời chúc chữ/giọng nói/video, huỷ đơn, đổi trả</t>
+          <t>Phiếu giao không in giá; testimonial; ngưỡng chống spam; KPI</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>🔴 Chặn go-live</t>
+          <t>🟡 Làm sau được</t>
         </is>
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>§14</t>
+          <t>§13</t>
         </is>
       </c>
       <c r="G97" s="9" t="inlineStr">
@@ -5009,7 +5033,7 @@
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>14.5</t>
+          <t>14.1</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
@@ -5019,13 +5043,13 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Chốt ngày go-live + người quyết định "đạt"</t>
+          <t>Gửi danh sách người dùng admin (email, vai trò admin/IT)</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr"/>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>🟠 Trước khi mở bán</t>
+          <t>🔴 Chặn go-live</t>
         </is>
       </c>
       <c r="F98" s="8" t="inlineStr">
@@ -5044,9 +5068,165 @@
       <c r="K98" s="9" t="n"/>
       <c r="L98" s="9" t="n"/>
     </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Phân công: nội dung, xử lý đơn, đổi trả/hoàn tiền, hỗ trợ khách</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr"/>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>🔴 Chặn go-live</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G99" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H99" s="9" t="n"/>
+      <c r="I99" s="10" t="n"/>
+      <c r="J99" s="10" t="n"/>
+      <c r="K99" s="9" t="n"/>
+      <c r="L99" s="9" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Tham dự buổi đào tạo /admin</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="inlineStr"/>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>🟠 Trước khi mở bán</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G100" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H100" s="9" t="n"/>
+      <c r="I100" s="10" t="n"/>
+      <c r="J100" s="10" t="n"/>
+      <c r="K100" s="9" t="n"/>
+      <c r="L100" s="9" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>UAT: thử đặt đơn thật đầu-cuối + ký biên bản nghiệm thu</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>COD + payOS, mua tặng với lời chúc chữ/giọng nói/video, huỷ đơn, đổi trả</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>🔴 Chặn go-live</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G101" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H101" s="9" t="n"/>
+      <c r="I101" s="10" t="n"/>
+      <c r="J101" s="10" t="n"/>
+      <c r="K101" s="9" t="n"/>
+      <c r="L101" s="9" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>14.5</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>Admin &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>Chốt ngày go-live + người quyết định "đạt"</t>
+        </is>
+      </c>
+      <c r="D102" s="8" t="inlineStr"/>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>🟠 Trước khi mở bán</t>
+        </is>
+      </c>
+      <c r="F102" s="8" t="inlineStr">
+        <is>
+          <t>§14</t>
+        </is>
+      </c>
+      <c r="G102" s="9" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="H102" s="9" t="n"/>
+      <c r="I102" s="10" t="n"/>
+      <c r="J102" s="10" t="n"/>
+      <c r="K102" s="9" t="n"/>
+      <c r="L102" s="9" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L98"/>
-  <conditionalFormatting sqref="G2:G98">
+  <autoFilter ref="A1:L102"/>
+  <conditionalFormatting sqref="G2:G102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Xong"</formula>
     </cfRule>
@@ -5060,16 +5240,16 @@
       <formula>"Bị chặn"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I98">
+  <conditionalFormatting sqref="I2:I102">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>AND($I2&lt;&gt;"",$I2&lt;TODAY(),$G2&lt;&gt;"Xong")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chưa bắt đầu,Đang làm,Chờ duyệt,Bị chặn,Xong"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:J98" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nhập ngày dạng dd/mm/yyyy" type="date" operator="greaterThan">
+    <dataValidation sqref="I2:J102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nhập ngày dạng dd/mm/yyyy" type="date" operator="greaterThan">
       <formula1>36526</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: protect router (ProtectedRoute/GuestRoute) và đưa ảnh fanpage vào web (D-106)
</commit_message>
<xml_diff>
--- a/docs/client-checklist/LAMVI-task-tracker-client.xlsx
+++ b/docs/client-checklist/LAMVI-task-tracker-client.xlsx
@@ -1547,14 +1547,18 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
       <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>14/10: đã thay logo trên menu/footer/đăng nhập/dashboard bằng logo fanpage (200px). Vẫn cần file vector gốc → xem 1.2</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -3391,14 +3395,18 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chờ duyệt</t>
         </is>
       </c>
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="10" t="n"/>
       <c r="J56" s="10" t="n"/>
       <c r="K56" s="9" t="n"/>
-      <c r="L56" s="9" t="n"/>
+      <c r="L56" s="9" t="inlineStr">
+        <is>
+          <t>14/10: đã đưa poster 5 đèn từ fanpage lên web (206px phóng lên, hơi mềm). Cần ảnh gốc + xác nhận quyền dùng</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">

</xml_diff>